<commit_message>
test: refresh formula qualification evidence
</commit_message>
<xml_diff>
--- a/demo/final cases/case_9_life_pricing/workbooks/case_9_life_pricing_incomplete.xlsx
+++ b/demo/final cases/case_9_life_pricing/workbooks/case_9_life_pricing_incomplete.xlsx
@@ -62,7 +62,7 @@
     <t xml:space="preserve">Published boundary</t>
   </si>
   <si>
-    <t xml:space="preserve">SUMPRODUCT and IRR are outside the current reconstruction catalogue and are retained verbatim.</t>
+    <t xml:space="preserve">IRR is outside the current reconstruction catalogue and is retained verbatim; SUMPRODUCT reconstructs independently.</t>
   </si>
   <si>
     <t xml:space="preserve">Expected internal result</t>
@@ -1672,7 +1672,7 @@
         <v>79</v>
       </c>
       <c r="B5" s="15" t="n">
-        <f aca="false">SUMPRODUCT(NetCashFlows,DiscountFactors)</f>
+        <f aca="false">SUMPRODUCT('Cash Flows'!$F$4:$F$9,'Cash Flows'!$G$4:$G$9)</f>
         <v>4599999.99927022</v>
       </c>
     </row>

</xml_diff>